<commit_message>
feat(gui): template + export xlsx avec colonnes TYPE SOURCE / SOURCE
_N_FIXED_COLS 10 -> 12 ; template régénéré avec les 2 en-têtes en tête.
Docstring module de validate.py corrigé (12 cols fixes A-L).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tapageur/gui/assets/template.xlsx
+++ b/tapageur/gui/assets/template.xlsx
@@ -841,7 +841,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA1"/>
+  <dimension ref="A1:AB1"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="33" customWidth="1" style="40" min="1" max="1"/>
@@ -873,139 +873,149 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
+          <t>TYPE SOURCE</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>SOURCE</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
           <t>INFO TAPEUR</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>DATE TAPAGE</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="E1" s="8" t="inlineStr">
         <is>
           <t>Date Émission Radio</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="F1" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">FESTOCHE
 EVENEMENT </t>
         </is>
       </c>
-      <c r="E1" s="8" t="inlineStr">
+      <c r="G1" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">STYLE 
 FESTOCHE / EVENEMENT </t>
         </is>
       </c>
-      <c r="F1" s="9" t="inlineStr">
+      <c r="H1" s="9" t="inlineStr">
         <is>
           <t>DATE</t>
         </is>
       </c>
-      <c r="G1" s="9" t="inlineStr">
+      <c r="I1" s="9" t="inlineStr">
         <is>
           <t>HEURE</t>
         </is>
       </c>
-      <c r="H1" s="9" t="inlineStr">
+      <c r="J1" s="10" t="inlineStr">
         <is>
           <t>LIEU</t>
         </is>
       </c>
-      <c r="I1" s="9" t="inlineStr">
+      <c r="K1" s="11" t="inlineStr">
         <is>
           <t>VILLE</t>
         </is>
       </c>
-      <c r="J1" s="10" t="inlineStr">
+      <c r="L1" s="12" t="inlineStr">
         <is>
           <t>PRIX</t>
         </is>
       </c>
-      <c r="K1" s="11" t="inlineStr">
+      <c r="M1" s="12" t="inlineStr">
         <is>
           <t>GENRE 1</t>
         </is>
       </c>
-      <c r="L1" s="12" t="inlineStr">
+      <c r="N1" s="13" t="inlineStr">
         <is>
           <t>NOM SPECTACLE 1 ( SV )</t>
         </is>
       </c>
-      <c r="M1" s="12" t="inlineStr">
+      <c r="O1" s="11" t="inlineStr">
         <is>
           <t>COMPAGNIE 1 ( SV ) ou
 GROUPE 1 / ARTISTE 1 ( C )</t>
         </is>
       </c>
-      <c r="N1" s="13" t="inlineStr">
+      <c r="P1" s="12" t="inlineStr">
         <is>
           <t>STYLE 
 SPECTACLE 1 (SV) / CONCERT 1 (C)</t>
         </is>
       </c>
-      <c r="O1" s="11" t="inlineStr">
+      <c r="Q1" s="12" t="inlineStr">
         <is>
           <t>GENRE 2</t>
         </is>
       </c>
-      <c r="P1" s="12" t="inlineStr">
+      <c r="R1" s="13" t="inlineStr">
         <is>
           <t>NOM SPECTACLE 2 ( SV )</t>
         </is>
       </c>
-      <c r="Q1" s="12" t="inlineStr">
+      <c r="S1" s="11" t="inlineStr">
         <is>
           <t>COMPAGNIE 2 ( SV ) ou
 GROUPE 2 / ARTISTE 2 ( C )</t>
         </is>
       </c>
-      <c r="R1" s="13" t="inlineStr">
+      <c r="T1" s="12" t="inlineStr">
         <is>
           <t>STYLE 
 SPECTACLE 2 ( SV ) / CONCERT 2 ( C )</t>
         </is>
       </c>
-      <c r="S1" s="11" t="inlineStr">
+      <c r="U1" s="12" t="inlineStr">
         <is>
           <t>GENRE 3</t>
         </is>
       </c>
-      <c r="T1" s="12" t="inlineStr">
+      <c r="V1" s="13" t="inlineStr">
         <is>
           <t>NOM SPECTACLE 3 ( SV )</t>
         </is>
       </c>
-      <c r="U1" s="12" t="inlineStr">
+      <c r="W1" s="11" t="inlineStr">
         <is>
           <t>COMPAGNIE 3 ( SV ) ou
 GROUPE 3 / ARTISTE 3 ( C )</t>
         </is>
       </c>
-      <c r="V1" s="13" t="inlineStr">
+      <c r="X1" s="12" t="inlineStr">
         <is>
           <t>STYLE 
 SPECTACLE 3 ( SV ) / CONCERT 3 ( C )</t>
         </is>
       </c>
-      <c r="W1" s="11" t="inlineStr">
+      <c r="Y1" s="12" t="inlineStr">
         <is>
           <t>GENRE 4</t>
         </is>
       </c>
-      <c r="X1" s="12" t="inlineStr">
+      <c r="Z1" s="13" t="inlineStr">
         <is>
           <t>NOM SPECTACLE 4 ( SV )</t>
         </is>
       </c>
-      <c r="Y1" s="12" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>COMPAGNIE 4 ( SV ) ou
 GROUPE 4 / ARTISTE 4 ( C )</t>
         </is>
       </c>
-      <c r="Z1" s="13" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>STYLE 
 SPECTACLE 4 ( SV ) / CONCERT 4 ( C )</t>

</xml_diff>

<commit_message>
fix(gui): décale aussi validations et largeurs du template (+2)
La régénération ne faisait que décaler les en-têtes de ligne 1 ; les listes
déroulantes (DATE/LIEU/VILLE/GENRE) et largeurs restaient sur les colonnes
d'origine, désalignées de 2 — régression sur la relecture. Régénère depuis
le template d'origine en décalant en-têtes + validations + largeurs, et
ajoute un test de non-régression.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tapageur/gui/assets/template.xlsx
+++ b/tapageur/gui/assets/template.xlsx
@@ -844,30 +844,34 @@
   <dimension ref="A1:AB1"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col width="33" customWidth="1" style="40" min="1" max="1"/>
-    <col width="29.75" customWidth="1" style="40" min="2" max="4"/>
+    <col width="18" customWidth="1" style="40" min="1" max="1"/>
+    <col width="30" customWidth="1" style="40" min="2" max="4"/>
+    <col width="33" customWidth="1" style="40" min="3" max="3"/>
+    <col width="29.75" customWidth="1" style="40" min="4" max="4"/>
     <col width="29.38" customWidth="1" style="40" min="5" max="5"/>
     <col width="28.5" customWidth="1" style="40" min="6" max="6"/>
-    <col width="28.25" customWidth="1" style="40" min="7" max="7"/>
-    <col width="39.25" customWidth="1" style="40" min="8" max="8"/>
-    <col width="31" customWidth="1" style="40" min="9" max="9"/>
-    <col width="33.5" customWidth="1" style="40" min="10" max="10"/>
-    <col width="33.38" customWidth="1" style="40" min="11" max="11"/>
-    <col width="38.88" customWidth="1" style="40" min="12" max="12"/>
-    <col width="42.75" customWidth="1" style="40" min="13" max="13"/>
-    <col width="43.75" customWidth="1" style="40" min="14" max="14"/>
-    <col width="34.38" customWidth="1" style="40" min="15" max="15"/>
-    <col width="32.75" customWidth="1" style="40" min="16" max="16"/>
-    <col width="34" customWidth="1" style="40" min="17" max="17"/>
-    <col width="28.38" customWidth="1" style="40" min="18" max="18"/>
-    <col width="38.5" customWidth="1" style="40" min="19" max="19"/>
-    <col width="30" customWidth="1" style="40" min="20" max="20"/>
-    <col width="45.13" customWidth="1" style="40" min="21" max="21"/>
-    <col width="54.13" customWidth="1" style="40" min="22" max="22"/>
-    <col width="43" customWidth="1" style="40" min="23" max="23"/>
-    <col width="39" customWidth="1" style="40" min="24" max="24"/>
-    <col width="41.63" customWidth="1" style="40" min="25" max="25"/>
-    <col width="42.5" customWidth="1" style="40" min="26" max="26"/>
+    <col width="29.38" customWidth="1" style="40" min="7" max="7"/>
+    <col width="28.5" customWidth="1" style="40" min="8" max="8"/>
+    <col width="28.25" customWidth="1" style="40" min="9" max="9"/>
+    <col width="39.25" customWidth="1" style="40" min="10" max="10"/>
+    <col width="31" customWidth="1" style="40" min="11" max="11"/>
+    <col width="33.5" customWidth="1" style="40" min="12" max="12"/>
+    <col width="33.38" customWidth="1" style="40" min="13" max="13"/>
+    <col width="38.88" customWidth="1" style="40" min="14" max="14"/>
+    <col width="42.75" customWidth="1" style="40" min="15" max="15"/>
+    <col width="43.75" customWidth="1" style="40" min="16" max="16"/>
+    <col width="34.38" customWidth="1" style="40" min="17" max="17"/>
+    <col width="32.75" customWidth="1" style="40" min="18" max="18"/>
+    <col width="34" customWidth="1" style="40" min="19" max="19"/>
+    <col width="28.38" customWidth="1" style="40" min="20" max="20"/>
+    <col width="38.5" customWidth="1" style="40" min="21" max="21"/>
+    <col width="30" customWidth="1" style="40" min="22" max="22"/>
+    <col width="45.13" customWidth="1" style="40" min="23" max="23"/>
+    <col width="54.13" customWidth="1" style="40" min="24" max="24"/>
+    <col width="43" customWidth="1" style="40" min="25" max="25"/>
+    <col width="39" customWidth="1" style="40" min="26" max="26"/>
+    <col width="41.63" customWidth="1" style="40" min="27" max="27"/>
+    <col width="42.5" customWidth="1" style="40" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1032,100 +1036,100 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="32">
-    <dataValidation sqref="H76:H101 H103:H106 H108 H110:H137" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="J76:J101 J103:J106 J108 J110:J137" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>salles_lieux!$A$1:$A216</formula1>
     </dataValidation>
-    <dataValidation sqref="H8:H13" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="J8:J13" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>salles_lieux!$A$1:$A208</formula1>
     </dataValidation>
-    <dataValidation sqref="I14:I15" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="K14:K15" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>communes!$A$1:$A385</formula1>
     </dataValidation>
-    <dataValidation sqref="H23:H37" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="J23:J37" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>salles_lieux!$A$1:$A226</formula1>
     </dataValidation>
-    <dataValidation sqref="H161:H164" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="J161:J164" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>salles_lieux!$A$1:$A298</formula1>
     </dataValidation>
-    <dataValidation sqref="H41:H43" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="J41:J43" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>salles_lieux!$A$1:$A201</formula1>
     </dataValidation>
-    <dataValidation sqref="I161:I164" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="K161:K164" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>communes!$A$1:$A468</formula1>
     </dataValidation>
-    <dataValidation sqref="I44:I64" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="K44:K64" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>communes!$A$1:$A375</formula1>
     </dataValidation>
-    <dataValidation sqref="H68:H72 H139:H141 H143:H153 H155:H157 H159:H160 H165:H181" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="J68:J72 J139:J141 J143:J153 J155:J157 J159:J160 J165:J181" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>salles_lieux!$A$1:$A206</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F182 F184:F1079" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H182 H184:H1079" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>date!$C$1:$C$32</formula1>
     </dataValidation>
-    <dataValidation sqref="H4:H7" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="J4:J7" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>salles_lieux!$A$1:$A203</formula1>
     </dataValidation>
-    <dataValidation sqref="H182 H184:H1079" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="J182 J184:J1079" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>salles_lieux!$A$1:$A314</formula1>
     </dataValidation>
-    <dataValidation sqref="H14:H15" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="J14:J15" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>salles_lieux!$A$1:$A215</formula1>
     </dataValidation>
-    <dataValidation sqref="H138" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="J138" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>salles_lieux!$A$1:$A279</formula1>
     </dataValidation>
-    <dataValidation sqref="I41:I43" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="K41:K43" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>communes!$A$1:$A371</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I3" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K3" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>communes!$A$1:$A370</formula1>
     </dataValidation>
-    <dataValidation sqref="I76:I137" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="K76:K137" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>communes!$A$1:$A386</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K80 K82:K1079 O2:O1079 S2:S1079 W2:W1079" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M80 M82:M1079 Q2:Q1079 U2:U1079 Y2:Y1079" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"c,sv"</formula1>
     </dataValidation>
-    <dataValidation sqref="I73:I75" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="K73:K75" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>communes!$A$1:$A382</formula1>
     </dataValidation>
-    <dataValidation sqref="I23:I37" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="K23:K37" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>communes!$A$1:$A396</formula1>
     </dataValidation>
-    <dataValidation sqref="H73:H75" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="J73:J75" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>salles_lieux!$A$1:$A212</formula1>
     </dataValidation>
-    <dataValidation sqref="H16:H22" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="J16:J22" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>salles_lieux!$A$1:$A218</formula1>
     </dataValidation>
-    <dataValidation sqref="I16:I22" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="K16:K22" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>communes!$A$1:$A388</formula1>
     </dataValidation>
-    <dataValidation sqref="H44:H64" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="J44:J64" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>salles_lieux!$A$1:$A205</formula1>
     </dataValidation>
-    <dataValidation sqref="I138" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="K138" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>communes!$A$1:$A449</formula1>
     </dataValidation>
-    <dataValidation sqref="I4:I7" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="K4:K7" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>communes!$A$1:$A373</formula1>
     </dataValidation>
-    <dataValidation sqref="I65:I72 I139:I160 I165:I181" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="K65:K72 K139:K160 K165:K181" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>communes!$A$1:$A373</formula1>
     </dataValidation>
-    <dataValidation sqref="I38:I40" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="K38:K40" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>communes!$A$1:$A413</formula1>
     </dataValidation>
-    <dataValidation sqref="I182:I1079" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="K182:K1079" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>communes!$A$1:$A484</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H3" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J3" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>salles_lieux!$A$1:$A200</formula1>
     </dataValidation>
-    <dataValidation sqref="H38:H40" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="J38:J40" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>salles_lieux!$A$1:$A243</formula1>
     </dataValidation>
-    <dataValidation sqref="I8:I13" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="K8:K13" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>communes!$A$1:$A378</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>